<commit_message>
Migrate ski-touring + la-skateparks articles; wire Magazine cards to articles
- Add ski-touring and guide-la-skateparks to the article-page template (all 5
  magazine articles now migrated; both reuse quote-pull grey-box + cards-profile)
- quote-pull: render quotation/attribution as authored — drop the added curly-quote
  glyphs and em-dash attribution prefix so it matches the source on every article
- cards-article: Magazine "All Articles" cards link to their migrated article pages
  (env-aware /content prefix, .html stripped); scoped to /magazine/ links only so
  unmigrated /adventures/ cards and dynamic Recent Articles stay '#'

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article-page.report.xlsx
+++ b/tools/importer/reports/import-article-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="72">
   <si>
     <t>_reportFile</t>
   </si>
@@ -166,6 +166,21 @@
     <t>https://wknd.site/us/en/magazine/arctic-surfing.html</t>
   </si>
   <si>
+    <t>us/en/magazine/guide-la-skateparks.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/guide-la-skateparks</t>
+  </si>
+  <si>
+    <t>2026-08-10T11:33:22.273Z</t>
+  </si>
+  <si>
+    <t>Ultimate Guide to LA Skateparks</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/guide-la-skateparks.html</t>
+  </si>
+  <si>
     <t>us/en/magazine/san-diego-surf.report.json</t>
   </si>
   <si>
@@ -182,6 +197,21 @@
   </si>
   <si>
     <t>https://wknd.site/us/en/magazine/san-diego-surf.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/ski-touring.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/ski-touring</t>
+  </si>
+  <si>
+    <t>2026-08-10T11:10:18.530Z</t>
+  </si>
+  <si>
+    <t>Ski Touring</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/ski-touring.html</t>
   </si>
   <si>
     <t>us/en/magazine/western-australia.report.json</t>
@@ -585,15 +615,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="46" customWidth="1"/>
+    <col min="1" max="1" width="48" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="28" customWidth="1"/>
+    <col min="7" max="7" width="33" customWidth="1"/>
     <col min="8" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
@@ -784,10 +814,10 @@
         <v>51</v>
       </c>
       <c r="B8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" t="s">
         <v>52</v>
-      </c>
-      <c r="C8" t="s">
-        <v>53</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
@@ -796,21 +826,21 @@
         <v>47</v>
       </c>
       <c r="F8" t="s">
+        <v>53</v>
+      </c>
+      <c r="G8" t="s">
         <v>54</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>55</v>
-      </c>
-      <c r="H8" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" t="s">
         <v>57</v>
-      </c>
-      <c r="B9" t="s">
-        <v>45</v>
       </c>
       <c r="C9" t="s">
         <v>58</v>
@@ -829,6 +859,58 @@
       </c>
       <c r="H9" t="s">
         <v>61</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>47</v>
+      </c>
+      <c r="F10" t="s">
+        <v>64</v>
+      </c>
+      <c r="G10" t="s">
+        <v>65</v>
+      </c>
+      <c r="H10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>47</v>
+      </c>
+      <c r="F11" t="s">
+        <v>69</v>
+      </c>
+      <c r="G11" t="s">
+        <v>70</v>
+      </c>
+      <c r="H11" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>